<commit_message>
Fondations v5 : assistant commercial (moteur), IA générative côté serveur, champs personnalisés, modèles d'e-mails
- Types et migration v5 : module Assistant, réglage IA (désactivé par défaut),
  champs personnalisés, modèles d'e-mails ; finances masquées sur un espace client neuf
- Moteur de l'assistant : score de risque explicable, prévision, rapport du matin,
  brouillons de relance à partir de modèles
- IA (Claude) uniquement côté serveur : clé ANTHROPIC_API_KEY, session, autorisation
  du directeur commercial, limitation des demandes, données minimisées

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LHM9bLdLjJgrdZ7pjFSNxV
</commit_message>
<xml_diff>
--- a/public/modeles/Configuration-CRM.xlsx
+++ b/public/modeles/Configuration-CRM.xlsx
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="110">
   <si>
     <t>Configuration de votre CRM</t>
   </si>
@@ -365,10 +365,13 @@
     <t>Activé</t>
   </si>
   <si>
+    <t>Assistant commercial</t>
+  </si>
+  <si>
+    <t>Oui</t>
+  </si>
+  <si>
     <t>Propositions commerciales</t>
-  </si>
-  <si>
-    <t>Oui</t>
   </si>
   <si>
     <t>Finances</t>
@@ -1009,28 +1012,28 @@
         <v>8</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>51</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -6538,7 +6541,14 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>87</v>
+      </c>
+    </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25"/>
@@ -7064,16 +7074,16 @@
         <v>42</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>33</v>
@@ -7082,13 +7092,13 @@
         <v>67</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25"/>
@@ -7636,25 +7646,25 @@
         <v>44</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>36</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25"/>

</xml_diff>